<commit_message>
- Maelle's corrections and real-world testing for Mardi - Standalone version
</commit_message>
<xml_diff>
--- a/output/planning_Mardi.xlsx
+++ b/output/planning_Mardi.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -468,7 +468,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Bar public 19:00-20:30</t>
+          <t>Ailes 19:00-20:30</t>
         </is>
       </c>
     </row>
@@ -483,59 +483,59 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Bar public 17:30-19:00; Abeilles Ruche 23:30-00:30</t>
+          <t>Déambule Goulus 16:30-18:00; Bar public 20:30-22:00 (**)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Alexandra</t>
+          <t>Alex</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Déambule Spoutnik 17:00-19:00</t>
+          <t>Bar loges 19:00-20:30; Entrée backstage 23:30-00:30</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Alice</t>
+          <t>Alexandra</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Ailes 18:00-20:00; Abeilles Ruche 22:00-23:30</t>
+          <t>Bar loges 22:00-23:30</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Analou</t>
+          <t>Alice</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Abeilles Ruche 19:00-20:30</t>
+          <t>Abeilles Ruche 15:45-17:30; Bar public 20:30-22:00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Anna</t>
+          <t>Ana-Lou</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -543,14 +543,14 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Bar loges 19:30-21:00</t>
+          <t>Abeilles Ruche 19:00-20:30</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Annouk</t>
+          <t>Andy</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -558,14 +558,14 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Bar public 16:00-17:30; Bar public 20:30-22:00</t>
+          <t>Bar public 17:30-19:00; Entrée backstage 22:00-23:30 (**)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Antonin</t>
+          <t>Anna</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -573,29 +573,29 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Abeilles Ruche 16:00-17:30; Bar public 22:00-23:30</t>
+          <t>Ailes 17:30-19:00; Bar public 22:00-23:30 (**)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Arsène</t>
+          <t>Annouk</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Entrée backstage 19:00-20:30</t>
+          <t>Déambule Gerry 16:30-18:00; Bar public 20:30-22:00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Arthur</t>
+          <t>Antonin</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -603,167 +603,175 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Déambule FBI 17:00-19:00; Bar loges 21:00-22:30</t>
+          <t>Déambule Goulus 20:00-21:30; Bar public 23:30-00:30</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Athénaé</t>
+          <t>Arsène</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Déambule Volkanik 16:30-18:30; Entrée backstage 20:30-22:00</t>
+          <t>Abeilles Ruche 19:00-20:30</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Auxence</t>
+          <t>Arthur</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Déambule Goulus 16:30-18:00</t>
+          <t>Bar public 19:00-20:30; Abeilles Ruche 23:30-00:30</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Ava</t>
+          <t>Athénaé</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Abeilles Ruche 20:30-22:00</t>
+          <t>Entrée backstage 17:30-19:00; Déambule Colbok 21:00-23:00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Benoît</t>
+          <t>Auxence</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Abeilles Ruche 15:45-17:30; Bar loges 20:30-22:00 (***)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Corentin</t>
+          <t>Ava</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Bar public 19:00-20:30; Bar public 23:30-00:30</t>
+          <t>Ailes 20:30-22:00</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Emma</t>
+          <t>Benoît</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2</v>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Abeilles Ruche 19:00-20:30; Abeilles Ruche 23:30-00:30</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="C17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Enzo</t>
+          <t>Corentin</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Ailes 20:00-22:00</t>
+          <t>Ailes 16:00-17:30; Bar public 20:30-22:00</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Eugénie</t>
+          <t>Emma</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C19" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Bar loges 17:30-19:00; Bar public 23:30-00:30</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Iris</t>
+          <t>Eugénie</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Bar public 16:00-17:30; Déambule Spoutnik 22:00-23:00</t>
+          <t>Bar loges 22:00-23:30</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Jamilah</t>
+          <t>Frank</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0</v>
-      </c>
-      <c r="C21" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Bar public 19:00-20:30; Bar loges 23:30-01:00</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Jolan</t>
+          <t>Iris</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Abeilles Ruche 20:30-22:00</t>
+          <t>Bar public 16:00-17:30; Ailes 20:30-22:00</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Jonas</t>
+          <t>Jamilah</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -774,22 +782,22 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Jules</t>
+          <t>Jolan</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Bar public 20:30-22:00</t>
+          <t>Déambule Goulus 16:30-18:00; Abeilles Ruche 20:30-22:00</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Julie</t>
+          <t>Jonas</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -800,33 +808,33 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Kristel</t>
+          <t>Jules</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>0</v>
-      </c>
-      <c r="C26" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Ailes 19:00-20:30</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Lisa J.</t>
+          <t>Julie</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2</v>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Abeilles Ruche 17:30-19:00; Ailes 22:00-24:00</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="C27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Lisa M.</t>
+          <t>Kristel</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -837,7 +845,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Louis C.</t>
+          <t>Lisa J.</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -845,40 +853,40 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Abeilles Ruche 17:30-19:00; Bar public 23:30-00:30</t>
+          <t>Abeilles Ruche 15:45-17:30; Déambule FBI 21:30-23:30</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Louis P.</t>
+          <t>Lisa M.</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>2</v>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Abeilles Ruche 17:30-19:00; Ailes 22:00-24:00</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="C30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Louise</t>
+          <t>Louis C.</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0</v>
-      </c>
-      <c r="C31" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Ailes 16:00-17:30; Déambule Gerry 20:30-22:00</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Lucas</t>
+          <t>Louis P.</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -886,29 +894,25 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Ailes 18:00-20:00; Bar public 22:00-23:30</t>
+          <t>Bar public 16:00-17:30; Entrée backstage 20:30-22:00 (***)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Lucie</t>
+          <t>Louise</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1</v>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Déambule Colbok 17:00-19:00</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="C33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Léa B.</t>
+          <t>Lucas</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -916,70 +920,70 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Entrée backstage 17:30-19:00; Bar public 22:00-23:30</t>
+          <t>Bar loges 19:00-20:30; Ailes 23:30-00:30</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Léa C.</t>
+          <t>Lucie</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>2</v>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Ailes 18:00-20:00; Ailes 22:00-24:00</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="C35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Marius</t>
+          <t>Léa B.</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0</v>
-      </c>
-      <c r="C36" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Déambule FBI 17:00-19:00; Déambule Spoutnik 22:00-23:00</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Marot</t>
+          <t>Léa C.</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Bar public 17:30-19:00; Bar loges 21:00-22:30</t>
+          <t>Bar public 17:30-19:00</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Mathis</t>
+          <t>Marius</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Bar loges 16:30-18:00; Tech Jacquard 21:00-23:00</t>
+          <t>Tech Phusis 18:00-19:30</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Matteo</t>
+          <t>Marot</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -987,55 +991,55 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Déambule Gerry 20:30-22:00</t>
+          <t>Ailes 22:00-23:30</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Maxime</t>
+          <t>Mathis</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0</v>
-      </c>
-      <c r="C40" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Abeilles Ruche 17:30-19:00; Ailes 22:00-23:30</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Maya</t>
+          <t>Matteo</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>2</v>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Ailes 16:00-18:00; Abeilles Ruche 20:30-22:00</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="C41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Maëlan</t>
+          <t>Maxime</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Ailes 16:00-18:00; Abeilles Ruche 22:00-23:30</t>
+          <t>Tech Jacquard 20:15-22:30</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Maëlle</t>
+          <t>Maya C.</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1043,29 +1047,29 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Bar public 17:30-19:00; Déambule FBI 21:30-23:30</t>
+          <t>Déambule Colbok 17:00-19:00; Abeilles Ruche 22:00-23:30</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Mickaël</t>
+          <t>Maya R.</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Ailes 20:00-22:00</t>
+          <t>Bar public 17:30-19:00; Abeilles Ruche 22:00-23:30</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Mireille</t>
+          <t>Maëlan</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1073,44 +1077,36 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Tech Phusis 18:00-19:30</t>
+          <t>Abeilles Ruche 19:00-20:30</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Morgana</t>
+          <t>Maëlle</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>2</v>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Tech PCGB 19:30-20:30; Bar loges 22:30-24:00</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="C46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Morgane</t>
+          <t>Mehdi</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>2</v>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Bar public 19:00-20:30; Bar loges 22:30-24:00</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="C47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Nathalia</t>
+          <t>Mickaël</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1118,40 +1114,44 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Abeilles Ruche 16:00-17:30; Déambule Goulus 20:00-21:30</t>
+          <t>Ailes 16:00-17:30; Déambule Goulus 20:00-21:30</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Noah</t>
+          <t>Mireille</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Abeilles Ruche 19:00-20:30</t>
+          <t>Ailes 17:30-19:00; Déambule Volkanik 22:30-24:00</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Patrick</t>
+          <t>Morgana</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>0</v>
-      </c>
-      <c r="C50" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Tech PCGB 19:30-20:30; Ailes 23:30-00:30</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Rama</t>
+          <t>Morgane</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1159,14 +1159,14 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Bar loges 18:00-19:30; Déambule Volkanik 22:30-24:00</t>
+          <t>Ailes 17:30-19:00; Bar public 22:00-23:30</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Raphaël</t>
+          <t>Nathalia</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1174,14 +1174,14 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Tech T'es rien… 17:00-18:30; Entrée backstage 22:00-23:30</t>
+          <t>Abeilles Ruche 17:30-19:00; Bar public 22:00-23:30</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Raphaëlle</t>
+          <t>Noah</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1189,55 +1189,51 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Bar public 19:00-20:30; Entrée backstage 23:30-00:30</t>
+          <t>Abeilles Ruche 17:30-19:00; Bar public 22:00-23:30</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Roxanne</t>
+          <t>Patrick</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>2</v>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Bar loges 18:00-19:30; Bar public 23:30-00:30</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="C54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Simon</t>
+          <t>Rama</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>2</v>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Bar public 16:00-17:30; Déambule Colbok 21:00-23:00</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="C55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Sébastien</t>
+          <t>Raphaël</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0</v>
-      </c>
-      <c r="C56" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Tech T'es rien… 17:00-18:30; Abeilles Ruche 22:00-23:30</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Theo</t>
+          <t>Raphaëlle</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1245,14 +1241,14 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Déambule Gerry 16:30-18:00; Bar public 20:30-22:00</t>
+          <t>Entrée backstage 19:00-20:30; Bar loges 23:30-01:00</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Thibault</t>
+          <t>Roxanne</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1260,14 +1256,14 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Entrée backstage 16:00-17:30; Déambule Goulus 20:00-21:30</t>
+          <t>Bar loges 16:00-17:30; Abeilles Ruche 20:30-22:00</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Titouan</t>
+          <t>Sacha</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1275,14 +1271,14 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Ailes 16:00-18:00; Bar public 20:30-22:00</t>
+          <t>Bar public 19:00-20:30; Abeilles Ruche 23:30-00:30</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Tristan</t>
+          <t>Simon</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1290,37 +1286,123 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Déambule Goulus 16:30-18:00; Ailes 20:00-22:00</t>
+          <t>Déambule Volkanik 16:30-18:30; Abeilles Ruche 20:30-22:00</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Yann</t>
+          <t>Sébastien</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>2</v>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Bar loges 16:30-18:00; Abeilles Ruche 22:00-23:30</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="C61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
+          <t>Theo</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>2</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Entrée backstage 15:45-17:30; Bar loges 20:30-22:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Thibault</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>2</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Bar public 19:00-20:30; Abeilles Ruche 23:30-00:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Tician</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>2</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Bar public 16:00-17:30; Ailes 20:30-22:00 (***)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Titouan</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>2</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Ailes 19:00-20:30; Bar public 23:30-00:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Tristan</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>2</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Bar loges 17:30-19:00; Ailes 22:00-23:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Yann</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>1</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Déambule Spoutnik 17:00-19:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
           <t>Ysatis</t>
         </is>
       </c>
-      <c r="B62" t="n">
-        <v>2</v>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Abeilles Ruche 16:00-17:30; Bar loges 19:30-21:00</t>
+      <c r="B68" t="n">
+        <v>2</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Bar loges 16:00-17:30; Ailes 23:30-00:30 (***)</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1392,7 +1474,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>15:45</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1411,7 +1493,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Antonin, Nathalia, Ysatis</t>
+          <t>Alice, Auxence, Lisa J.</t>
         </is>
       </c>
     </row>
@@ -1442,7 +1524,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Lisa J., Louis C., Louis P.</t>
+          <t>Mathis, Nathalia, Noah</t>
         </is>
       </c>
     </row>
@@ -1473,7 +1555,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Analou, Emma, Noah</t>
+          <t>Ana-Lou, Arsène, Maëlan</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1586,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Ava, Jolan, Maya</t>
+          <t>Jolan, Roxanne, Simon</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1617,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Alice, Maëlan, Yann</t>
+          <t>Maya C., Raphaël, Maya R.</t>
         </is>
       </c>
     </row>
@@ -1556,17 +1638,17 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Alegria Lily, Emma</t>
+          <t>Arthur, Thibault, Sacha</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1665,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -1597,7 +1679,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Maëlan, Maya, Titouan</t>
+          <t>Corentin, Louis C., Mickaël</t>
         </is>
       </c>
     </row>
@@ -1609,12 +1691,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1628,7 +1710,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Alice, Léa C., Lucas</t>
+          <t>Anna, Mireille, Morgane</t>
         </is>
       </c>
     </row>
@@ -1640,12 +1722,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -1659,7 +1741,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Enzo, Mickaël, Tristan</t>
+          <t>Agathe, Jules, Titouan</t>
         </is>
       </c>
     </row>
@@ -1671,12 +1753,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
           <t>22:00</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>24:00</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -1690,69 +1772,69 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Léa C., Lisa J., Louis P.</t>
+          <t>Ava, Iris, Tician (***)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Bar loges</t>
+          <t>Ailes</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Mathis, Yann</t>
+          <t>Marot, Mathis, Tristan</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Bar loges</t>
+          <t>Ailes</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Rama, Roxanne</t>
+          <t>Lucas, Morgana, Ysatis (***)</t>
         </is>
       </c>
     </row>
@@ -1764,12 +1846,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1783,7 +1865,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Anna, Ysatis</t>
+          <t>Roxanne, Ysatis</t>
         </is>
       </c>
     </row>
@@ -1795,12 +1877,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>22:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1814,7 +1896,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Arthur, Marot</t>
+          <t>Emma, Tristan</t>
         </is>
       </c>
     </row>
@@ -1826,12 +1908,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>22:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>24:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1845,100 +1927,100 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Morgana, Morgane</t>
+          <t>Lucas, Alex</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Bar public</t>
+          <t>Bar loges</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Annouk, Iris, Simon</t>
+          <t>Auxence (***), Theo</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Bar public</t>
+          <t>Bar loges</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Alegria Lily, Maëlle, Marot</t>
+          <t>Alexandra, Eugénie</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Bar public</t>
+          <t>Bar loges</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>01:00</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E19" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Agathe, Corentin, Morgane, Raphaëlle</t>
+          <t>Raphaëlle, Frank</t>
         </is>
       </c>
     </row>
@@ -1950,26 +2032,26 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Annouk, Jules, Theo, Titouan</t>
+          <t>Iris, Louis P., Tician</t>
         </is>
       </c>
     </row>
@@ -1981,12 +2063,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -2000,7 +2082,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Antonin, Léa B., Lucas</t>
+          <t>Andy, Léa C., Maya R.</t>
         </is>
       </c>
     </row>
@@ -2012,119 +2094,119 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>00:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F22" t="n">
         <v>0</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Corentin, Louis C., Roxanne</t>
+          <t>Arthur, Thibault, Frank, Sacha</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Entrée backstage</t>
+          <t>Bar public</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Thibault</t>
+          <t>Alegria Lily (**), Alice, Annouk, Corentin</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Entrée backstage</t>
+          <t>Bar public</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E24" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Léa B.</t>
+          <t>Anna (**), Morgane, Nathalia, Noah</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Entrée backstage</t>
+          <t>Bar public</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F25" t="n">
         <v>0</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Arsène</t>
+          <t>Antonin, Emma, Titouan</t>
         </is>
       </c>
     </row>
@@ -2136,12 +2218,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>15:45</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -2155,7 +2237,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Athénaé</t>
+          <t>Theo</t>
         </is>
       </c>
     </row>
@@ -2167,12 +2249,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -2186,7 +2268,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Raphaël</t>
+          <t>Athénaé</t>
         </is>
       </c>
     </row>
@@ -2198,12 +2280,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>00:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -2224,17 +2306,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Déambule Gerry</t>
+          <t>Entrée backstage</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -2248,24 +2330,24 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Theo</t>
+          <t>Louis P. (***)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Déambule Gerry</t>
+          <t>Entrée backstage</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -2279,24 +2361,24 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Matteo</t>
+          <t>Andy (**)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Déambule Colbok</t>
+          <t>Entrée backstage</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -2310,24 +2392,24 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Lucie</t>
+          <t>Alex</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Déambule Colbok</t>
+          <t>Déambule Gerry</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -2341,86 +2423,86 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Simon</t>
+          <t>Annouk</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Déambule Goulus</t>
+          <t>Déambule Gerry</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F33" t="n">
         <v>0</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Auxence, Tristan</t>
+          <t>Louis C.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Déambule Goulus</t>
+          <t>Déambule Colbok</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F34" t="n">
         <v>0</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Nathalia, Thibault</t>
+          <t>Maya C.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Déambule Volkanik</t>
+          <t>Déambule Colbok</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -2441,79 +2523,79 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Déambule Volkanik</t>
+          <t>Déambule Goulus</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>22:30</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>24:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F36" t="n">
         <v>0</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Rama</t>
+          <t>Alegria Lily, Jolan</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Déambule Spoutnik</t>
+          <t>Déambule Goulus</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F37" t="n">
         <v>0</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Alexandra</t>
+          <t>Antonin, Mickaël</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Déambule Spoutnik</t>
+          <t>Déambule Volkanik</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -2527,24 +2609,24 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Iris</t>
+          <t>Simon</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Déambule FBI</t>
+          <t>Déambule Volkanik</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>22:30</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>24:00</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -2558,24 +2640,24 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Arthur</t>
+          <t>Mireille</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Déambule FBI</t>
+          <t>Déambule Spoutnik</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -2589,19 +2671,19 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Maëlle</t>
+          <t>Yann</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Tech Jacquard</t>
+          <t>Déambule Spoutnik</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2620,24 +2702,24 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Mathis</t>
+          <t>Léa B.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Tech PCGB</t>
+          <t>Déambule FBI</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -2651,24 +2733,24 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Morgana</t>
+          <t>Léa B.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Tech T'es rien…</t>
+          <t>Déambule FBI</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -2682,7 +2764,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Raphaël</t>
+          <t>Lisa J.</t>
         </is>
       </c>
     </row>
@@ -2713,28 +2795,121 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Mireille</t>
+          <t>Marius</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>(**) Personne affectée malgré un blocage de priorité 1</t>
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Tech Jacquard</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>1</v>
+      </c>
+      <c r="E45" t="n">
+        <v>1</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Maxime</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>(*) Personne affectée malgré une préférence de blocage (priorité 2)</t>
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Tech PCGB</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Morgana</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>(***) Personne affectée malgré une préférence de blocage (priorité 3)</t>
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Tech T'es rien…</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Raphaël</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>(*) Personne affectée malgré un blocage de priorité 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>(**) Personne affectée malgré un blocage de priorité 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>(***) Personne affectée malgré un blocage de priorité 3</t>
         </is>
       </c>
     </row>
@@ -2749,7 +2924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2783,154 +2958,154 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Rotation Déambule/tardif manquante</t>
+          <t>Préférence non respectée (priorité 2)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Entrée backstage</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>22:00-23:30</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Anna n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
+          <t>Andy avait indiqué une préférence (priorité 2) sur ce créneau (Lorde)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Rotation Déambule/tardif manquante</t>
+          <t>Préférence non respectée (priorité 2)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Bar public</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>20:30-22:00</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Annouk n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
+          <t>Alegria Lily avait indiqué une préférence (priorité 2) sur ce créneau (Lorde)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Rotation Déambule/tardif manquante</t>
+          <t>Préférence non respectée (priorité 2)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Bar public</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>22:00-23:30</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Enzo n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
+          <t>Anna avait indiqué une préférence (priorité 2) sur ce créneau (Lorde)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rotation Déambule/tardif manquante</t>
+          <t>Préférence non respectée (priorité 3)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Entrée backstage</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>20:30-22:00</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Jolan n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
+          <t>Louis P. avait indiqué une préférence (priorité 3) sur ce créneau (Lorde)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Rotation Déambule/tardif manquante</t>
+          <t>Préférence non respectée (priorité 3)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Bar loges</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>20:30-22:00</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Marot n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
+          <t>Auxence avait indiqué une préférence (priorité 3) sur ce créneau (Lorde)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Rotation Déambule/tardif manquante</t>
+          <t>Préférence non respectée (priorité 3)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Ailes</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>23:30-00:30</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Mathis n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
+          <t>Ysatis avait indiqué une préférence (priorité 3) sur ce créneau (Asaf Avidan)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Rotation Déambule/tardif manquante</t>
+          <t>Préférence non respectée (priorité 3)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Ailes</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>20:30-22:00</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Maya n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
+          <t>Tician avait indiqué une préférence (priorité 3) sur ce créneau (Lorde)</t>
         </is>
       </c>
     </row>
@@ -2952,7 +3127,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Mickaël n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
+          <t>Alice n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
         </is>
       </c>
     </row>
@@ -2974,7 +3149,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Mireille n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
+          <t>Auxence n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
         </is>
       </c>
     </row>
@@ -2996,7 +3171,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Noah n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
+          <t>Corentin n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
         </is>
       </c>
     </row>
@@ -3018,7 +3193,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Titouan n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
+          <t>Iris n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
         </is>
       </c>
     </row>
@@ -3040,14 +3215,14 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Ysatis n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
+          <t>Julie n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Shifts incomplets</t>
+          <t>Rotation Déambule/tardif manquante</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -3062,14 +3237,14 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Alexandra n'a fait que 1 shift(s) sur 2 attendus</t>
+          <t>Léa C. n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Shifts incomplets</t>
+          <t>Rotation Déambule/tardif manquante</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3084,14 +3259,14 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Anna n'a fait que 1 shift(s) sur 2 attendus</t>
+          <t>Lisa M. n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Shifts incomplets</t>
+          <t>Rotation Déambule/tardif manquante</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3106,14 +3281,14 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Auxence n'a fait que 1 shift(s) sur 2 attendus</t>
+          <t>Louis P. n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Shifts incomplets</t>
+          <t>Rotation Déambule/tardif manquante</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3128,14 +3303,14 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Enzo n'a fait que 1 shift(s) sur 2 attendus</t>
+          <t>Maëlan n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Shifts incomplets</t>
+          <t>Rotation Déambule/tardif manquante</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3150,14 +3325,14 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Jolan n'a fait que 1 shift(s) sur 2 attendus</t>
+          <t>Maëlle n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Shifts incomplets</t>
+          <t>Rotation Déambule/tardif manquante</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3172,14 +3347,14 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Lucie n'a fait que 1 shift(s) sur 2 attendus</t>
+          <t>Marius n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Shifts incomplets</t>
+          <t>Rotation Déambule/tardif manquante</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3194,14 +3369,14 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Matteo n'a fait que 1 shift(s) sur 2 attendus</t>
+          <t>Maxime n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Shifts incomplets</t>
+          <t>Rotation Déambule/tardif manquante</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3216,14 +3391,14 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Mickaël n'a fait que 1 shift(s) sur 2 attendus</t>
+          <t>Roxanne n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Shifts incomplets</t>
+          <t>Rotation Déambule/tardif manquante</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3238,29 +3413,95 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Mireille n'a fait que 1 shift(s) sur 2 attendus</t>
+          <t>Theo n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>Rotation Déambule/tardif manquante</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Tician n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Rotation Déambule/tardif manquante</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Mehdi n'a encore eu aucun créneau Déambule ou tardif cette semaine</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>Shifts incomplets</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Noah n'a fait que 1 shift(s) sur 2 attendus</t>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Maëlan n'a fait que 1 shift(s) sur 2 attendus</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Shifts incomplets</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Yann n'a fait que 1 shift(s) sur 2 attendus</t>
         </is>
       </c>
     </row>

</xml_diff>